<commit_message>
Actulizando general proyecto + fase 3 completa - Pendiente nestor
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias Documentación/Sprint 4/Impediment Backlog Proyecto Stockify - Sprint 4.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias Documentación/Sprint 4/Impediment Backlog Proyecto Stockify - Sprint 4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\b5m\Downloads\Capstone_2025_Grupo8-main\Fase 2\Evidencias Proyecto\Evidencias Documentación\Sprint 4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\b5m\Downloads\Capstone_2025_Grupo8-main_ULTIMAPRESENTACION\Capstone_2025_Grupo8-main\Fase 2\Evidencias Proyecto\Evidencias Documentación\Sprint 4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA9E789-A1FB-4A9A-87BF-96AEFA24D1BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB59558-7195-4FA6-A450-3E4F0455D9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3870" yWindow="2625" windowWidth="21600" windowHeight="10830" xr2:uid="{5D59AC23-7906-42B4-A607-2B72F4503BB1}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5D59AC23-7906-42B4-A607-2B72F4503BB1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1138,7 +1138,7 @@
     </row>
     <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>51</v>
@@ -1164,7 +1164,7 @@
     </row>
     <row r="19" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>54</v>
@@ -1190,7 +1190,7 @@
     </row>
     <row r="20" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>57</v>
@@ -1216,7 +1216,7 @@
     </row>
     <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>59</v>

</xml_diff>